<commit_message>
data: apply Task 5 case corrections and refresh evaluation outputs
- raw/case: PLUS1_003 now the live 2026-09-03 factory (ANTARA-sourced),
  PLUS1_005 splits the reported vs conditional investment, RETURN_002
  demotes the unsupported "orders returned to China" claim
- processed/case_database_v0.1 + metadata/evidence_cases_v0.1 rebuilt;
  evidence index grows to 28 rows (NEWS_024/025, NEWS_017 flagged dead)
- evaluation/* recomputed: Task 3 P@5 0.913 / R@10 0.810 / EA 0.929,
  Task 4 0.940 / 0.827, Task 6/7 unchanged
</commit_message>
<xml_diff>
--- a/data/evaluation/benchmark_results.xlsx
+++ b/data/evaluation/benchmark_results.xlsx
@@ -1261,10 +1261,10 @@
         </is>
       </c>
       <c r="F12" s="2" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G12" s="2" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H12" s="2" t="n">
         <v>2</v>
@@ -1295,12 +1295,12 @@
       </c>
       <c r="O12" s="2" t="inlineStr">
         <is>
-          <t>NEWS_015</t>
+          <t>NEWS_015; NEWS_024; NEWS_025</t>
         </is>
       </c>
       <c r="P12" s="2" t="inlineStr">
         <is>
-          <t>待观察（建设中）</t>
+          <t>成功（已投产并转为全本地生产）</t>
         </is>
       </c>
     </row>
@@ -1436,7 +1436,7 @@
       </c>
       <c r="P14" s="2" t="inlineStr">
         <is>
-          <t>待观察（计划阶段）</t>
+          <t>待观察（计划阶段；投资金额需拆分核实）</t>
         </is>
       </c>
     </row>
@@ -1576,7 +1576,7 @@
       </c>
       <c r="P16" s="2" t="inlineStr">
         <is>
-          <t>局部回流（未完全放弃印度）</t>
+          <t>工程团队撤回（订单/产能回流中国为待验证推断，未完全放弃印度）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: move Task 5 cases out of the ingest path (held-out benchmark)
- data/raw/case/*.md -> data/evaluation/case_benchmark/case/*.md
- data/metadata/evidence_cases_v0.1.xlsx ->
  data/evaluation/case_benchmark/evidence_cases_v0.1.xlsx
- registry rebuilt for 30 Task 1 evidence docs only
- evaluation outputs refreshed (Task 2/3/4/5/6/7)
</commit_message>
<xml_diff>
--- a/data/evaluation/benchmark_results.xlsx
+++ b/data/evaluation/benchmark_results.xlsx
@@ -11,7 +11,7 @@
     <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Case Results'!$A$1:$P$18</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Case Results'!$A$1:$N$18</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -431,25 +431,23 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:N18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="44" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
-    <col width="32" customWidth="1" min="11" max="11"/>
-    <col width="34" customWidth="1" min="12" max="12"/>
-    <col width="12" customWidth="1" min="13" max="13"/>
-    <col width="12" customWidth="1" min="14" max="14"/>
-    <col width="20" customWidth="1" min="15" max="15"/>
-    <col width="26" customWidth="1" min="16" max="16"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="46" customWidth="1" min="5" max="5"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="24" customWidth="1" min="8" max="8"/>
+    <col width="32" customWidth="1" min="9" max="9"/>
+    <col width="34" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="42" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -470,65 +468,55 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
+          <t>case_type</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
           <t>decision_problem</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>case_doc_id</t>
-        </is>
-      </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>case_doc_rank_baseline</t>
+          <t>benchmark_held_out</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>case_doc_rank_optimized</t>
+          <t>expected_decision_type</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>company_docs_in_corpus</t>
+          <t>evidence_index_ids</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">
         <is>
-          <t>company_docs_retrieved</t>
+          <t>expected_risks</t>
         </is>
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>company_doc_recall</t>
+          <t>risks_identified_baseline</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>expected_risks</t>
+          <t>risk_recall_baseline</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
         <is>
-          <t>risks_identified_baseline</t>
+          <t>risk_recall_optimized</t>
         </is>
       </c>
       <c r="M1" s="1" t="inlineStr">
         <is>
-          <t>risk_recall_baseline</t>
+          <t>policy_evidence_top5_baseline</t>
         </is>
       </c>
       <c r="N1" s="1" t="inlineStr">
-        <is>
-          <t>risk_recall_optimized</t>
-        </is>
-      </c>
-      <c r="O1" s="1" t="inlineStr">
-        <is>
-          <t>source_articles</t>
-        </is>
-      </c>
-      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>verdict</t>
         </is>
@@ -552,53 +540,51 @@
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
+          <t>China → Southeast Asia relocation</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
           <t>比亚迪 正在评估将部分产能从中国转移至泰国。管理层应基于现有证据判断该决策的风险。</t>
         </is>
       </c>
-      <c r="E2" s="2" t="inlineStr">
-        <is>
-          <t>RELOC_001</t>
-        </is>
-      </c>
-      <c r="F2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H2" s="2" t="n">
-        <v>2</v>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>多地区混合布局</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_001</t>
+        </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
         <is>
-          <t>PLUS1_003; RELOC_001</t>
-        </is>
-      </c>
-      <c r="J2" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K2" s="2" t="inlineStr">
-        <is>
           <t>Market Access Risk; Political Risk; Trade Risk</t>
         </is>
       </c>
-      <c r="L2" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="N2" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="O2" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_001</t>
-        </is>
-      </c>
-      <c r="P2" s="2" t="inlineStr">
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="L2" s="2" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>TRD_001; MOFCOM_001; TRD_003; CASE_004; CASE_001</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
         <is>
           <t>成功（本地供应链仍依赖中国）</t>
         </is>
@@ -622,53 +608,51 @@
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
+          <t>China → Southeast Asia relocation</t>
+        </is>
+      </c>
+      <c r="E3" s="2" t="inlineStr">
+        <is>
           <t>长安汽车 正在评估将部分产能从中国转移至泰国。管理层应基于现有证据判断该决策的风险。</t>
         </is>
       </c>
-      <c r="E3" s="2" t="inlineStr">
-        <is>
-          <t>RELOC_002</t>
-        </is>
-      </c>
-      <c r="F3" s="2" t="n">
+      <c r="F3" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G3" s="2" t="inlineStr">
+        <is>
+          <t>多地区混合布局</t>
+        </is>
+      </c>
+      <c r="H3" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_002; COMPANY_REPORT_001</t>
+        </is>
+      </c>
+      <c r="I3" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="J3" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G3" s="2" t="n">
+      <c r="L3" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I3" s="2" t="inlineStr">
-        <is>
-          <t>RELOC_002</t>
-        </is>
-      </c>
-      <c r="J3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K3" s="2" t="inlineStr">
-        <is>
-          <t>Market Access Risk; Operational Risk; Trade Risk</t>
-        </is>
-      </c>
-      <c r="L3" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M3" s="2" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="N3" s="2" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="O3" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_002; COMPANY_REPORT_001</t>
-        </is>
-      </c>
-      <c r="P3" s="2" t="inlineStr">
+      <c r="M3" s="2" t="inlineStr">
+        <is>
+          <t>TRD_001; MOFCOM_001; TRD_003; CASE_004; CASE_001</t>
+        </is>
+      </c>
+      <c r="N3" s="2" t="inlineStr">
         <is>
           <t>成功（早期，产能爬坡中）</t>
         </is>
@@ -692,53 +676,51 @@
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
+          <t>China → Southeast Asia relocation</t>
+        </is>
+      </c>
+      <c r="E4" s="2" t="inlineStr">
+        <is>
           <t>国轩高科 正在评估将部分产能从中国转移至越南。管理层应基于现有证据判断该决策的风险。</t>
         </is>
       </c>
-      <c r="E4" s="2" t="inlineStr">
-        <is>
-          <t>RELOC_003</t>
-        </is>
-      </c>
-      <c r="F4" s="2" t="n">
+      <c r="F4" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G4" s="2" t="inlineStr">
+        <is>
+          <t>多地区混合布局</t>
+        </is>
+      </c>
+      <c r="H4" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_003; NEWS_004</t>
+        </is>
+      </c>
+      <c r="I4" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="J4" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G4" s="2" t="n">
+      <c r="L4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I4" s="2" t="inlineStr">
-        <is>
-          <t>RELOC_003</t>
-        </is>
-      </c>
-      <c r="J4" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K4" s="2" t="inlineStr">
-        <is>
-          <t>Market Access Risk; Supply Chain Risk; Trade Risk</t>
-        </is>
-      </c>
-      <c r="L4" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M4" s="2" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="N4" s="2" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="O4" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_003; NEWS_004</t>
-        </is>
-      </c>
-      <c r="P4" s="2" t="inlineStr">
+      <c r="M4" s="2" t="inlineStr">
+        <is>
+          <t>TRD_001; TRD_003; MOFCOM_001; CASE_001; CASE_008</t>
+        </is>
+      </c>
+      <c r="N4" s="2" t="inlineStr">
         <is>
           <t>成功（材料端仍依赖中国）</t>
         </is>
@@ -762,53 +744,51 @@
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
+          <t>China → Southeast Asia relocation</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
           <t>亿纬锂能 正在评估将部分产能从中国转移至马来西亚。管理层应基于现有证据判断该决策的风险。</t>
         </is>
       </c>
-      <c r="E5" s="2" t="inlineStr">
-        <is>
-          <t>RELOC_004</t>
-        </is>
-      </c>
-      <c r="F5" s="2" t="n">
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>多地区混合布局</t>
+        </is>
+      </c>
+      <c r="H5" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_005</t>
+        </is>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>Operational Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G5" s="2" t="n">
+      <c r="L5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I5" s="2" t="inlineStr">
-        <is>
-          <t>RELOC_004</t>
-        </is>
-      </c>
-      <c r="J5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk; Trade Risk</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk; Trade Risk</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="N5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="O5" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_005</t>
-        </is>
-      </c>
-      <c r="P5" s="2" t="inlineStr">
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>TRD_001; TRD_003; CASE_007; MOFCOM_001; CASE_001</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
         <is>
           <t>成功（爬坡中）</t>
         </is>
@@ -832,53 +812,51 @@
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
+          <t>China → Southeast Asia relocation</t>
+        </is>
+      </c>
+      <c r="E6" s="2" t="inlineStr">
+        <is>
           <t>欣旺达 正在评估将部分产能从中国转移至越南。管理层应基于现有证据判断该决策的风险。</t>
         </is>
       </c>
-      <c r="E6" s="2" t="inlineStr">
-        <is>
-          <t>RELOC_005</t>
-        </is>
-      </c>
-      <c r="F6" s="2" t="n">
+      <c r="F6" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G6" s="2" t="inlineStr">
+        <is>
+          <t>多地区混合布局</t>
+        </is>
+      </c>
+      <c r="H6" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_006; NEWS_007</t>
+        </is>
+      </c>
+      <c r="I6" s="2" t="inlineStr">
+        <is>
+          <t>Operational Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="J6" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G6" s="2" t="n">
+      <c r="L6" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I6" s="2" t="inlineStr">
-        <is>
-          <t>RELOC_005</t>
-        </is>
-      </c>
-      <c r="J6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K6" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk; Trade Risk</t>
-        </is>
-      </c>
-      <c r="L6" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M6" s="2" t="n">
-        <v>0.667</v>
-      </c>
-      <c r="N6" s="2" t="n">
-        <v>0.667</v>
-      </c>
-      <c r="O6" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_006; NEWS_007</t>
-        </is>
-      </c>
-      <c r="P6" s="2" t="inlineStr">
+      <c r="M6" s="2" t="inlineStr">
+        <is>
+          <t>TRD_001; TRD_003; MOFCOM_001; CASE_001; CASE_008</t>
+        </is>
+      </c>
+      <c r="N6" s="2" t="inlineStr">
         <is>
           <t>待观察（尚未投产）</t>
         </is>
@@ -902,53 +880,51 @@
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
+          <t>China → Southeast Asia relocation</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="inlineStr">
+        <is>
           <t>蜂巢能源 正在评估将部分产能从中国转移至泰国。管理层应基于现有证据判断该决策的风险。</t>
         </is>
       </c>
-      <c r="E7" s="2" t="inlineStr">
-        <is>
-          <t>RELOC_006</t>
-        </is>
-      </c>
-      <c r="F7" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G7" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H7" s="2" t="n">
-        <v>2</v>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr">
+        <is>
+          <t>多地区混合布局</t>
+        </is>
+      </c>
+      <c r="H7" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_008</t>
+        </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
         <is>
-          <t>RELOC_006; RETURN_004</t>
-        </is>
-      </c>
-      <c r="J7" s="2" t="n">
+          <t>Market Access Risk; Operational Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="J7" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K7" s="2" t="inlineStr">
-        <is>
-          <t>Market Access Risk; Operational Risk; Trade Risk</t>
-        </is>
-      </c>
-      <c r="L7" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M7" s="2" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="N7" s="2" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="O7" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_008</t>
-        </is>
-      </c>
-      <c r="P7" s="2" t="inlineStr">
+      <c r="L7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>TRD_001; MOFCOM_001; TRD_003; CASE_001; CASE_004</t>
+        </is>
+      </c>
+      <c r="N7" s="2" t="inlineStr">
         <is>
           <t>成功（局部环节外移）</t>
         </is>
@@ -972,53 +948,51 @@
       </c>
       <c r="D8" s="2" t="inlineStr">
         <is>
+          <t>China → Southeast Asia relocation</t>
+        </is>
+      </c>
+      <c r="E8" s="2" t="inlineStr">
+        <is>
           <t>华友钴业 正在评估将部分产能从中国转移至印尼。管理层应基于现有证据判断该决策的风险。</t>
         </is>
       </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>RELOC_007</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H8" s="2" t="n">
-        <v>1</v>
+      <c r="F8" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G8" s="2" t="inlineStr">
+        <is>
+          <t>多地区混合布局</t>
+        </is>
+      </c>
+      <c r="H8" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_009</t>
+        </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
         <is>
-          <t>RELOC_007</t>
-        </is>
-      </c>
-      <c r="J8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K8" s="2" t="inlineStr">
-        <is>
           <t>Political Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M8" s="2" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="N8" s="2" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="O8" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_009</t>
-        </is>
-      </c>
-      <c r="P8" s="2" t="inlineStr">
+      <c r="J8" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K8" s="2" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="L8" s="2" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="M8" s="2" t="inlineStr">
+        <is>
+          <t>MOFCOM_001; TRD_001; CASE_001; TRD_003; CASE_008</t>
+        </is>
+      </c>
+      <c r="N8" s="2" t="inlineStr">
         <is>
           <t>成功（上游外移，加工仍在国内）</t>
         </is>
@@ -1042,53 +1016,51 @@
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
+          <t>China → Southeast Asia relocation</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="inlineStr">
+        <is>
           <t>中伟股份 正在评估将部分产能从中国转移至印尼。管理层应基于现有证据判断该决策的风险。</t>
         </is>
       </c>
-      <c r="E9" s="2" t="inlineStr">
-        <is>
-          <t>RELOC_008</t>
-        </is>
-      </c>
-      <c r="F9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H9" s="2" t="n">
-        <v>1</v>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr">
+        <is>
+          <t>多地区混合布局</t>
+        </is>
+      </c>
+      <c r="H9" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_010; NEWS_011</t>
+        </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
         <is>
-          <t>RELOC_008</t>
-        </is>
-      </c>
-      <c r="J9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K9" s="2" t="inlineStr">
-        <is>
           <t>Operational Risk; Political Risk; Supply Chain Risk</t>
         </is>
       </c>
-      <c r="L9" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M9" s="2" t="n">
+      <c r="J9" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K9" s="2" t="n">
         <v>0.667</v>
       </c>
-      <c r="N9" s="2" t="n">
+      <c r="L9" s="2" t="n">
         <v>0.667</v>
       </c>
-      <c r="O9" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_010; NEWS_011</t>
-        </is>
-      </c>
-      <c r="P9" s="2" t="inlineStr">
+      <c r="M9" s="2" t="inlineStr">
+        <is>
+          <t>TRD_001; MOFCOM_001; CASE_001; TRD_003; CASE_008</t>
+        </is>
+      </c>
+      <c r="N9" s="2" t="inlineStr">
         <is>
           <t>成功（上游外移）</t>
         </is>
@@ -1112,53 +1084,51 @@
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
+          <t>China + 1 strategy</t>
+        </is>
+      </c>
+      <c r="E10" s="2" t="inlineStr">
+        <is>
           <t>宁德时代 正在推进 China+1 布局（匈牙利）。管理层应基于现有证据评估该布局的风险。</t>
         </is>
       </c>
-      <c r="E10" s="2" t="inlineStr">
-        <is>
-          <t>PLUS1_001</t>
-        </is>
-      </c>
-      <c r="F10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H10" s="2" t="n">
-        <v>2</v>
+      <c r="F10" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G10" s="2" t="inlineStr">
+        <is>
+          <t>多地区混合布局</t>
+        </is>
+      </c>
+      <c r="H10" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_012; NEWS_013</t>
+        </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
         <is>
-          <t>PLUS1_001; PLUS1_002</t>
-        </is>
-      </c>
-      <c r="J10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
           <t>Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N10" s="2" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="O10" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_012; NEWS_013</t>
-        </is>
-      </c>
-      <c r="P10" s="2" t="inlineStr">
+      <c r="J10" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K10" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L10" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M10" s="2" t="inlineStr">
+        <is>
+          <t>CASE_010; CASE_008; CASE_001; CASE_004; CASE_007</t>
+        </is>
+      </c>
+      <c r="N10" s="2" t="inlineStr">
         <is>
           <t>待观察（试生产中，投资周期长）</t>
         </is>
@@ -1182,53 +1152,51 @@
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
+          <t>China + 1 strategy</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="inlineStr">
+        <is>
           <t>宁德时代 正在推进 China+1 布局（印尼）。管理层应基于现有证据评估该布局的风险。</t>
         </is>
       </c>
-      <c r="E11" s="2" t="inlineStr">
-        <is>
-          <t>PLUS1_002</t>
-        </is>
-      </c>
-      <c r="F11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H11" s="2" t="n">
-        <v>2</v>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr">
+        <is>
+          <t>多地区混合布局</t>
+        </is>
+      </c>
+      <c r="H11" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_014</t>
+        </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
         <is>
-          <t>PLUS1_001; PLUS1_002</t>
-        </is>
-      </c>
-      <c r="J11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K11" s="2" t="inlineStr">
-        <is>
           <t>Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
-      <c r="L11" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M11" s="2" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="N11" s="2" t="n">
-        <v>0.25</v>
-      </c>
-      <c r="O11" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_014</t>
-        </is>
-      </c>
-      <c r="P11" s="2" t="inlineStr">
+      <c r="J11" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K11" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="L11" s="2" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="M11" s="2" t="inlineStr">
+        <is>
+          <t>CASE_010; CASE_008; CASE_001; CASE_004; CASE_007</t>
+        </is>
+      </c>
+      <c r="N11" s="2" t="inlineStr">
         <is>
           <t>待观察（建设中）</t>
         </is>
@@ -1252,53 +1220,51 @@
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
+          <t>China + 1 strategy</t>
+        </is>
+      </c>
+      <c r="E12" s="2" t="inlineStr">
+        <is>
           <t>比亚迪 正在推进 China+1 布局（印尼）。管理层应基于现有证据评估该布局的风险。</t>
         </is>
       </c>
-      <c r="E12" s="2" t="inlineStr">
-        <is>
-          <t>PLUS1_003</t>
-        </is>
-      </c>
-      <c r="F12" s="2" t="n">
+      <c r="F12" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G12" s="2" t="inlineStr">
+        <is>
+          <t>多地区混合布局</t>
+        </is>
+      </c>
+      <c r="H12" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_015; NEWS_024; NEWS_025</t>
+        </is>
+      </c>
+      <c r="I12" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="J12" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G12" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H12" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="I12" s="2" t="inlineStr">
-        <is>
-          <t>PLUS1_003; RELOC_001</t>
-        </is>
-      </c>
-      <c r="J12" s="2" t="n">
+      <c r="L12" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="K12" s="2" t="inlineStr">
-        <is>
-          <t>Market Access Risk; Operational Risk; Trade Risk</t>
-        </is>
-      </c>
-      <c r="L12" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M12" s="2" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="N12" s="2" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="O12" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_015; NEWS_024; NEWS_025</t>
-        </is>
-      </c>
-      <c r="P12" s="2" t="inlineStr">
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>CASE_010; CASE_008; CASE_001; CASE_004; WH_002</t>
+        </is>
+      </c>
+      <c r="N12" s="2" t="inlineStr">
         <is>
           <t>成功（已投产并转为全本地生产）</t>
         </is>
@@ -1322,49 +1288,51 @@
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
+          <t>China + 1 strategy</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="inlineStr">
+        <is>
           <t>晶科能源 正在推进 China+1 布局（马来西亚 / 越南 / 美国）。管理层应基于现有证据评估该布局的风险。</t>
         </is>
       </c>
-      <c r="E13" s="2" t="inlineStr">
-        <is>
-          <t>PLUS1_004</t>
-        </is>
-      </c>
-      <c r="F13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="H13" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I13" s="2" t="inlineStr"/>
-      <c r="J13" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="K13" s="2" t="inlineStr">
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr">
+        <is>
+          <t>多地区混合布局</t>
+        </is>
+      </c>
+      <c r="H13" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_016</t>
+        </is>
+      </c>
+      <c r="I13" s="2" t="inlineStr">
         <is>
           <t>Market Access Risk; Political Risk; Regulatory Risk; Trade Risk</t>
         </is>
       </c>
-      <c r="L13" s="2" t="inlineStr">
-        <is>
-          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
-        </is>
-      </c>
-      <c r="M13" s="2" t="n">
+      <c r="J13" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K13" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="N13" s="2" t="n">
+      <c r="L13" s="2" t="n">
         <v>0.5</v>
       </c>
-      <c r="O13" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_016</t>
-        </is>
-      </c>
-      <c r="P13" s="2" t="inlineStr">
+      <c r="M13" s="2" t="inlineStr">
+        <is>
+          <t>CASE_010; CASE_003; TRD_001; WH_002; TRD_003</t>
+        </is>
+      </c>
+      <c r="N13" s="2" t="inlineStr">
         <is>
           <t>成功（多地产能分散风险）</t>
         </is>
@@ -1388,53 +1356,51 @@
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
+          <t>China + 1 strategy</t>
+        </is>
+      </c>
+      <c r="E14" s="2" t="inlineStr">
+        <is>
           <t>三星电子 正在推进 China+1 布局（韩国 / 越南）。管理层应基于现有证据评估该布局的风险。</t>
         </is>
       </c>
-      <c r="E14" s="2" t="inlineStr">
-        <is>
-          <t>PLUS1_005</t>
-        </is>
-      </c>
-      <c r="F14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="G14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="H14" s="2" t="n">
-        <v>1</v>
+      <c r="F14" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G14" s="2" t="inlineStr">
+        <is>
+          <t>多地区混合布局</t>
+        </is>
+      </c>
+      <c r="H14" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_017</t>
+        </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
         <is>
-          <t>PLUS1_005</t>
-        </is>
-      </c>
-      <c r="J14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K14" s="2" t="inlineStr">
-        <is>
           <t>Operational Risk; Political Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
-      <c r="L14" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M14" s="2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="N14" s="2" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="O14" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_017</t>
-        </is>
-      </c>
-      <c r="P14" s="2" t="inlineStr">
+      <c r="J14" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K14" s="2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="L14" s="2" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="M14" s="2" t="inlineStr">
+        <is>
+          <t>CASE_010; CASE_001; CASE_008; TRD_003; TRD_001</t>
+        </is>
+      </c>
+      <c r="N14" s="2" t="inlineStr">
         <is>
           <t>待观察（计划阶段；投资金额需拆分核实）</t>
         </is>
@@ -1458,53 +1424,51 @@
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
+          <t>Reconsideration / Return to China</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="inlineStr">
+        <is>
           <t>恩捷股份 正在重新评估海外布局，考虑提高中国生产比例、收缩海外新增产能。管理层应基于现有证据评估这一调整的风险。</t>
         </is>
       </c>
-      <c r="E15" s="2" t="inlineStr">
-        <is>
-          <t>RETURN_001</t>
-        </is>
-      </c>
-      <c r="F15" s="2" t="n">
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr">
+        <is>
+          <t>提高中国生产比例</t>
+        </is>
+      </c>
+      <c r="H15" s="2" t="inlineStr">
+        <is>
+          <t>COMPANY_FILING_001; NEWS_018</t>
+        </is>
+      </c>
+      <c r="I15" s="2" t="inlineStr">
+        <is>
+          <t>Operational Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="J15" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="G15" s="2" t="n">
+      <c r="L15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="H15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="I15" s="2" t="inlineStr">
-        <is>
-          <t>RETURN_001</t>
-        </is>
-      </c>
-      <c r="J15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk; Trade Risk</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="n">
-        <v>0.667</v>
-      </c>
-      <c r="N15" s="2" t="n">
-        <v>0.667</v>
-      </c>
-      <c r="O15" s="2" t="inlineStr">
-        <is>
-          <t>COMPANY_FILING_001; NEWS_018</t>
-        </is>
-      </c>
-      <c r="P15" s="2" t="inlineStr">
+      <c r="M15" s="2" t="inlineStr">
+        <is>
+          <t>CASE_001; CASE_010; TRD_003; CASE_004; CASE_008</t>
+        </is>
+      </c>
+      <c r="N15" s="2" t="inlineStr">
         <is>
           <t>主动止损（成功止损，但海外布局目标未达成）</t>
         </is>
@@ -1528,53 +1492,51 @@
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
+          <t>Reconsideration / Return to China</t>
+        </is>
+      </c>
+      <c r="E16" s="2" t="inlineStr">
+        <is>
           <t>富士康 正在重新评估海外布局，考虑提高中国生产比例、收缩海外新增产能。管理层应基于现有证据评估这一调整的风险。</t>
         </is>
       </c>
-      <c r="E16" s="2" t="inlineStr">
-        <is>
-          <t>RETURN_002</t>
-        </is>
-      </c>
-      <c r="F16" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G16" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H16" s="2" t="n">
-        <v>1</v>
+      <c r="F16" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G16" s="2" t="inlineStr">
+        <is>
+          <t>提高中国生产比例</t>
+        </is>
+      </c>
+      <c r="H16" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_019; NEWS_020</t>
+        </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
         <is>
-          <t>RETURN_002</t>
-        </is>
-      </c>
-      <c r="J16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K16" s="2" t="inlineStr">
-        <is>
           <t>Operational Risk; Political Risk; Supply Chain Risk</t>
         </is>
       </c>
-      <c r="L16" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M16" s="2" t="n">
+      <c r="J16" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K16" s="2" t="n">
         <v>0.667</v>
       </c>
-      <c r="N16" s="2" t="n">
+      <c r="L16" s="2" t="n">
         <v>0.667</v>
       </c>
-      <c r="O16" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_019; NEWS_020</t>
-        </is>
-      </c>
-      <c r="P16" s="2" t="inlineStr">
+      <c r="M16" s="2" t="inlineStr">
+        <is>
+          <t>CASE_001; CASE_010; TRD_003; CASE_004; CASE_008</t>
+        </is>
+      </c>
+      <c r="N16" s="2" t="inlineStr">
         <is>
           <t>工程团队撤回（订单/产能回流中国为待验证推断，未完全放弃印度）</t>
         </is>
@@ -1598,53 +1560,51 @@
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
+          <t>Reconsideration / Return to China</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="inlineStr">
+        <is>
           <t>制造业外迁企业（行业层面） 正在重新评估海外布局，考虑提高中国生产比例、收缩海外新增产能。管理层应基于现有证据评估这一调整的风险。</t>
         </is>
       </c>
-      <c r="E17" s="2" t="inlineStr">
-        <is>
-          <t>RETURN_003</t>
-        </is>
-      </c>
-      <c r="F17" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G17" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H17" s="2" t="n">
-        <v>1</v>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr">
+        <is>
+          <t>提高中国生产比例</t>
+        </is>
+      </c>
+      <c r="H17" s="2" t="inlineStr">
+        <is>
+          <t>REUTERS_001; NEWS_023</t>
+        </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
         <is>
-          <t>RETURN_003</t>
-        </is>
-      </c>
-      <c r="J17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K17" s="2" t="inlineStr">
-        <is>
           <t>Operational Risk; Political Risk; Supply Chain Risk</t>
         </is>
       </c>
-      <c r="L17" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M17" s="2" t="n">
+      <c r="J17" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="n">
         <v>0.667</v>
       </c>
-      <c r="N17" s="2" t="n">
+      <c r="L17" s="2" t="n">
         <v>0.667</v>
       </c>
-      <c r="O17" s="2" t="inlineStr">
-        <is>
-          <t>REUTERS_001; NEWS_023</t>
-        </is>
-      </c>
-      <c r="P17" s="2" t="inlineStr">
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>CASE_001; WH_002; TRD_003; CASE_010; CASE_008</t>
+        </is>
+      </c>
+      <c r="N17" s="2" t="inlineStr">
         <is>
           <t>行业性回流（结构性调整，非全面逆转）</t>
         </is>
@@ -1668,60 +1628,58 @@
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
+          <t>Reconsideration / Return to China</t>
+        </is>
+      </c>
+      <c r="E18" s="2" t="inlineStr">
+        <is>
           <t>蜂巢能源 正在重新评估海外布局，考虑提高中国生产比例、收缩海外新增产能。管理层应基于现有证据评估这一调整的风险。</t>
         </is>
       </c>
-      <c r="E18" s="2" t="inlineStr">
-        <is>
-          <t>RETURN_004</t>
-        </is>
-      </c>
-      <c r="F18" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="G18" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="H18" s="2" t="n">
-        <v>2</v>
+      <c r="F18" s="2" t="inlineStr">
+        <is>
+          <t>是（未进入 RAG 语料）</t>
+        </is>
+      </c>
+      <c r="G18" s="2" t="inlineStr">
+        <is>
+          <t>维持现有海外布局（收缩新增）</t>
+        </is>
+      </c>
+      <c r="H18" s="2" t="inlineStr">
+        <is>
+          <t>NEWS_021; NEWS_022</t>
+        </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
         <is>
-          <t>RELOC_006; RETURN_004</t>
-        </is>
-      </c>
-      <c r="J18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="K18" s="2" t="inlineStr">
-        <is>
           <t>Operational Risk; Political Risk; Trade Risk</t>
         </is>
       </c>
-      <c r="L18" s="2" t="inlineStr">
-        <is>
-          <t>Operational Risk; Supply Chain Risk</t>
-        </is>
-      </c>
-      <c r="M18" s="2" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="N18" s="2" t="n">
-        <v>0.333</v>
-      </c>
-      <c r="O18" s="2" t="inlineStr">
-        <is>
-          <t>NEWS_021; NEWS_022</t>
-        </is>
-      </c>
-      <c r="P18" s="2" t="inlineStr">
+      <c r="J18" s="2" t="inlineStr">
+        <is>
+          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+        </is>
+      </c>
+      <c r="K18" s="2" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="L18" s="2" t="n">
+        <v>0.667</v>
+      </c>
+      <c r="M18" s="2" t="inlineStr">
+        <is>
+          <t>CASE_001; CASE_010; TRD_003; CASE_004; CASE_008</t>
+        </is>
+      </c>
+      <c r="N18" s="2" t="inlineStr">
         <is>
           <t>失败/主动退出（止损）</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:P18"/>
+  <autoFilter ref="A1:N18"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1732,12 +1690,12 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="34" customWidth="1" min="1" max="1"/>
     <col width="14" customWidth="1" min="2" max="2"/>
-    <col width="76" customWidth="1" min="3" max="3"/>
+    <col width="92" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -1775,56 +1733,56 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>case-document recall@5</t>
+          <t>held out of the RAG corpus</t>
         </is>
       </c>
       <c r="B3" s="2" t="n">
-        <v>0.9409999999999999</v>
+        <v>17</v>
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>案例自己的语料文档是否进入 Top-5</t>
+          <t>17/17 案例仅供评测，不进入知识库（避免答案泄漏）</t>
         </is>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>case-document recall@10</t>
+          <t>RAG corpus size</t>
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>0.9409999999999999</v>
+        <v>30</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>同上，Top-10</t>
+          <t>语料只含 Task 1 证据，不含任何 benchmark 案例</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>company-document recall@10</t>
+          <t>risk recall (baseline)</t>
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.9409999999999999</v>
+        <v>0.779</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>该案例所属企业在语料中的所有文档被召回的比例</t>
+          <t>见 Task 6：期望风险中被检索证据覆盖的比例</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>risk recall (baseline)</t>
+          <t>risk recall (optimized)</t>
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.461</v>
+        <v>0.779</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
@@ -1833,35 +1791,20 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr">
-        <is>
-          <t>risk recall (optimized)</t>
-        </is>
-      </c>
-      <c r="B7" s="2" t="n">
-        <v>0.461</v>
-      </c>
-      <c r="C7" s="2" t="inlineStr">
-        <is>
-          <t>见 Task 6</t>
-        </is>
-      </c>
+      <c r="A7" s="2" t="n"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" s="2" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="inlineStr">
+      <c r="A8" s="2" t="inlineStr">
         <is>
           <t>口径说明</t>
         </is>
       </c>
-      <c r="B9" s="2" t="inlineStr"/>
-      <c r="C9" s="2" t="inlineStr">
-        <is>
-          <t>案例绑定的 NEWS_* 是源文章（Task 5 Evidence Index），不在 RAG 语料中，因此不作为检索 gold；检索 gold 用案例自己在语料中的文档（= case_id）</t>
+      <c r="B8" s="2" t="inlineStr"/>
+      <c r="C8" s="2" t="inlineStr">
+        <is>
+          <t>本 benchmark 的案例是 held-out 答案键，故意不在 RAG 语料中，因此不再计算「案例文档召回」。检索层能力由 Task 2/3/4 评价，风险识别由 Task 6 评价；端到端「决策是否正确」需要 Agent 生成层，属下一阶段。</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
data: Task 1 v0.8 evidence workbook, EU/US originals, refreshed evaluation
Adds evidence_battery_EV_screened_v0.8.xlsx (36 rows = v0.7's 30 plus four
EU regulations and two US rules) together with the downloaded originals in
data/raw/policy/ so every row stays traceable.  The registry is rebuilt from
the v0.8 workbook and both US rows now use the "US" country code like the
rest of the corpus.

All evaluation outputs are regenerated against the 36-document corpus.
</commit_message>
<xml_diff>
--- a/data/evaluation/benchmark_results.xlsx
+++ b/data/evaluation/benchmark_results.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; MOFCOM_001; TRD_003; CASE_004; CASE_001</t>
+          <t>EU_003; TRD_001; CASE_001; CASE_004; MOFCOM_001</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -645,11 +645,11 @@
         <v>1</v>
       </c>
       <c r="L3" s="2" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; MOFCOM_001; TRD_003; CASE_004; CASE_001</t>
+          <t>TRD_001; CASE_004; CASE_001; MOFCOM_001; TRD_003</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -713,11 +713,11 @@
         <v>1</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; TRD_003; MOFCOM_001; CASE_001; CASE_008</t>
+          <t>TRD_001; TRD_003; CASE_001; MOFCOM_001; CASE_008</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K5" s="2" t="n">
@@ -785,7 +785,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; TRD_003; CASE_007; MOFCOM_001; CASE_001</t>
+          <t>TRD_001; TRD_003; CASE_007; CASE_001; CASE_010</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; TRD_003; MOFCOM_001; CASE_001; CASE_008</t>
+          <t>TRD_001; TRD_003; CASE_001; MOFCOM_001; CASE_008</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -917,11 +917,11 @@
         <v>1</v>
       </c>
       <c r="L7" s="2" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; MOFCOM_001; TRD_003; CASE_001; CASE_004</t>
+          <t>TRD_001; CASE_004; CASE_001; MOFCOM_001; TRD_003</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>MOFCOM_001; TRD_001; CASE_001; TRD_003; CASE_008</t>
+          <t>TRD_001; CASE_001; MOFCOM_001; CASE_008; CASE_004</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; MOFCOM_001; CASE_001; TRD_003; CASE_008</t>
+          <t>TRD_001; CASE_001; MOFCOM_001; CASE_008; CASE_004</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>CASE_010; CASE_008; CASE_001; CASE_004; WH_002</t>
+          <t>CASE_010; CASE_008; CASE_001; CASE_004; EU_003</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1318,7 +1318,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K13" s="2" t="n">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>CASE_010; CASE_003; TRD_001; WH_002; TRD_003</t>
+          <t>CASE_010; CASE_003; TRD_001; CASE_007; WH_002</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>CASE_010; CASE_001; CASE_008; TRD_003; TRD_001</t>
+          <t>CASE_010; CASE_008; CASE_001; CASE_003; CASE_004</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_010; TRD_003; CASE_004; CASE_008</t>
+          <t>CASE_001; CASE_010; CASE_008; CASE_004; EU_003</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1522,18 +1522,18 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K16" s="2" t="n">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0.667</v>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_010; TRD_003; CASE_004; CASE_008</t>
+          <t>CASE_001; CASE_010; CASE_008; CASE_004; CNGOV_001</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1590,18 +1590,18 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K17" s="2" t="n">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>0.667</v>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; WH_002; TRD_003; CASE_010; CASE_008</t>
+          <t>CASE_001; EU_003; CASE_010; CASE_008; CNGOV_001</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -1669,7 +1669,7 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_010; TRD_003; CASE_004; CASE_008</t>
+          <t>CASE_001; CASE_010; CASE_008; CASE_004; EU_003</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>30</v>
+        <v>36</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -1767,7 +1767,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.779</v>
+        <v>0.819</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.779</v>
+        <v>0.721</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data: Task 1 v0.9 evidence workbook, company/WTO/WB/DHS/IEA originals, refreshed evaluation
Adds evidence_battery_EV_screened_v0.9.xlsx (49 records; v0.8's 36 rows are
byte-identical) plus the originals it points at: SEC filings for Tesla, NIO,
XPeng, Li Auto and Albemarle under data/raw/company/, WTO India TPR and
Indonesia TPR, the WTO India tariff profile, USMCA Chapter 4, World Bank
LPI 2023, the DHS UFLPA notice, IEA Global EV Outlook 2025 and the SNE
Research release.

Also refreshes evidence_metadata_v0.1.json (49 entries) and every Task 2-7
artefact produced by the re-run.
</commit_message>
<xml_diff>
--- a/data/evaluation/benchmark_results.xlsx
+++ b/data/evaluation/benchmark_results.xlsx
@@ -581,7 +581,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>EU_003; TRD_001; CASE_001; CASE_004; MOFCOM_001</t>
+          <t>SNE_001; TRD_001; EU_003; CASE_001; MOFCOM_001</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -649,7 +649,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; CASE_004; CASE_001; MOFCOM_001; TRD_003</t>
+          <t>TRD_001; TRD_003; CASE_004; CASE_001; MOFCOM_001</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -717,7 +717,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; TRD_003; CASE_001; MOFCOM_001; CASE_008</t>
+          <t>TRD_001; TRD_003; MOFCOM_001; CASE_001; WB_001</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -774,7 +774,7 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Operational Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K5" s="2" t="n">
@@ -785,7 +785,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; TRD_003; CASE_007; CASE_001; CASE_010</t>
+          <t>TRD_001; TRD_003; CASE_007; WB_001; CASE_001</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -853,7 +853,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; TRD_003; CASE_001; MOFCOM_001; CASE_008</t>
+          <t>TRD_001; TRD_003; MOFCOM_001; CASE_001; WB_001</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -921,7 +921,7 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; CASE_004; CASE_001; MOFCOM_001; TRD_003</t>
+          <t>TRD_001; MOFCOM_001; CASE_001; CASE_004; TRD_003</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -989,7 +989,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; CASE_001; MOFCOM_001; CASE_008; CASE_004</t>
+          <t>TRD_001; WB_001; MOFCOM_001; CASE_001; CASE_008</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1057,7 +1057,7 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; CASE_001; MOFCOM_001; CASE_008; CASE_004</t>
+          <t>TRD_001; WB_001; CASE_001; MOFCOM_001; CASE_008</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>CASE_010; CASE_008; CASE_001; CASE_004; CASE_007</t>
+          <t>SNE_001; CASE_010; CASE_001; CASE_008; WH_002</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>CASE_010; CASE_008; CASE_001; CASE_004; CASE_007</t>
+          <t>SNE_001; CASE_010; CASE_001; CASE_008; TSLA_001</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>CASE_010; CASE_008; CASE_001; CASE_004; EU_003</t>
+          <t>SNE_001; CASE_010; CASE_008; CASE_001; EU_003</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1329,7 +1329,7 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>CASE_010; CASE_003; TRD_001; CASE_007; WH_002</t>
+          <t>CASE_010; CASE_003; TRD_001; WH_002; CASE_007</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>CASE_010; CASE_008; CASE_001; CASE_003; CASE_004</t>
+          <t>CASE_010; CASE_008; CASE_001; CASE_003; SNE_001</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1454,18 +1454,18 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K15" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L15" s="2" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_010; CASE_008; CASE_004; EU_003</t>
+          <t>CASE_001; DHS_001; CASE_008; CASE_004; EU_003</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1522,18 +1522,18 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K16" s="2" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="L16" s="2" t="n">
         <v>0.667</v>
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_010; CASE_008; CASE_004; CNGOV_001</t>
+          <t>DHS_001; CASE_001; CASE_008; CASE_004; EU_003</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1590,18 +1590,18 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K17" s="2" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>0.667</v>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; EU_003; CASE_010; CASE_008; CNGOV_001</t>
+          <t>CASE_001; DHS_001; EU_003; SNE_001; CASE_010</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -1658,18 +1658,18 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K18" s="2" t="n">
         <v>0.667</v>
       </c>
       <c r="L18" s="2" t="n">
-        <v>0.667</v>
+        <v>0.333</v>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; CASE_010; CASE_008; CASE_004; EU_003</t>
+          <t>CASE_001; DHS_001; CASE_008; CASE_004; EU_003</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>36</v>
+        <v>49</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -1767,7 +1767,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.819</v>
+        <v>0.779</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.721</v>
+        <v>0.681</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
data(task5): real evidence bindings for the 17 held-out cases + isolation audit
* case_database_v0.1.xlsx: related_evidence_ids now resolve to the 49-doc evidence
  base (was NEWS_*/REUTERS_* placeholders), plus external_source_refs and a
  per-case binding rationale; Evidence Index gains used_by_cases
* historical_case_benchmark.xlsx: Benchmark sheet carries related_evidence_ids /
  evidence_rationale / external_source_refs; QA registers the held-out audit,
  the 4 background-level overlaps and the RETURN_002 same-wire-story note
* case_benchmark/: the 17 narratives and the audit workbook follow the new fields
* re-ran the Task 6/7 writers and evaluation_report.md
</commit_message>
<xml_diff>
--- a/data/evaluation/benchmark_results.xlsx
+++ b/data/evaluation/benchmark_results.xlsx
@@ -560,7 +560,7 @@
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>NEWS_001</t>
+          <t>TRD_001; EU_003; IEA_001; CASE_004; WB_001</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -628,7 +628,7 @@
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>NEWS_002; COMPANY_REPORT_001</t>
+          <t>TRD_001; CASE_004; IEA_001; WB_001</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -696,7 +696,7 @@
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>NEWS_003; NEWS_004</t>
+          <t>TRD_001; TRD_003; SNE_001; WB_001; CASE_007</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -764,7 +764,7 @@
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>NEWS_005</t>
+          <t>TRD_001; TRD_003; CASE_007; SNE_001; WB_001</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -832,7 +832,7 @@
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>NEWS_006; NEWS_007</t>
+          <t>TRD_001; TRD_003; CASE_007; SNE_001; WB_001</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -900,7 +900,7 @@
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>NEWS_008</t>
+          <t>TRD_001; CASE_004; EU_003; IEA_001; WB_001</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -968,7 +968,7 @@
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>NEWS_009</t>
+          <t>WTO_004; TRD_003; SNE_001; WB_001</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -1036,7 +1036,7 @@
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>NEWS_010; NEWS_011</t>
+          <t>WTO_004; TRD_003; SNE_001; WB_001</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -1104,7 +1104,7 @@
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>NEWS_012; NEWS_013</t>
+          <t>EU_003; EU_001; EU_004; EU_002; SNE_001; IEA_001</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1172,7 +1172,7 @@
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>NEWS_014</t>
+          <t>WTO_004; TRD_003; SNE_001; IEA_001</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1240,7 +1240,7 @@
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>NEWS_015; NEWS_024; NEWS_025</t>
+          <t>WTO_004; IEA_001; SNE_001; TRD_003; EU_003</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1308,7 +1308,7 @@
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>NEWS_016</t>
+          <t>DOC_001; CASE_002; CASE_003; TRD_002</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1376,7 +1376,7 @@
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>NEWS_017</t>
+          <t>UNCTAD_001; TRD_003; WB_001; IMF_001</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1444,7 +1444,7 @@
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>COMPANY_FILING_001; NEWS_018</t>
+          <t>CASE_001; TRD_003; WB_001; SNE_001</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1512,7 +1512,7 @@
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>NEWS_019; NEWS_020</t>
+          <t>UNCTAD_001; WTO_002; WTO_003; CASE_001</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1580,7 +1580,7 @@
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>REUTERS_001; NEWS_023</t>
+          <t>CASE_001; WB_001; TRD_001; KPMG_001</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1648,7 +1648,7 @@
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>NEWS_021; NEWS_022</t>
+          <t>EU_003; EU_001; EU_004; CASE_001</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">

</xml_diff>

<commit_message>
data(task1): v0.9.2 —— MOFCOM_003–006 国别指南入库（49 → 53 篇 / 14,957 chunk）
- 新增 4 个原始文件：data/raw/policy/MOFCOM_003–006.pdf
  商务部《对外投资合作国别（地区）指南》越南 / 马来西亚 / 印度 / 泰国（2025 年版），
  合计 451 页 / 654 chunk；S 级官方报告。
- data/metadata/evidence_battery_EV_screened_v0.9.xlsx：sources 49 → 53 行，
  task1_annotations 同步 49 → 53 行，task1_status 追记 v0.9.2（含 uncertainty/可复现性）。
- data/metadata/evidence_metadata_v0.1.json：由 xlsx 重新派生（53 条）。
- data/vector_database/README.md：规模更新为 53 篇 / 14,957 chunk。
- 全链路重测产物：retrieval_questions / retrieval_results / entity_accuracy /
  baseline_report / risk_assessment_checklist / evidence_quality_test /
  historical_case_benchmark / benchmark_results / task4 / optimized /
  evaluation_report；case_database 的 QA 文本同步（53 条证据库、CASE_001 吸引子 13/17）。

关键结果：Task 6 risk_dimension missing 3 → 0（Risk Recall 1.000）；
43 题 P@5 0.763 / R@10 0.905 / EA 0.936。
</commit_message>
<xml_diff>
--- a/data/evaluation/benchmark_results.xlsx
+++ b/data/evaluation/benchmark_results.xlsx
@@ -570,18 +570,18 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K2" s="2" t="n">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="L2" s="2" t="n">
         <v>0.667</v>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>SNE_001; EU_003; TRD_001; CASE_001; MOFCOM_001</t>
+          <t>SNE_001; EU_003; TRD_001; MOFCOM_003; CASE_004</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
@@ -638,7 +638,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K3" s="2" t="n">
@@ -649,7 +649,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; TRD_003; CASE_001; CASE_004; MOFCOM_001</t>
+          <t>TRD_001; MOFCOM_003; CASE_004; TRD_003; NIO_001</t>
         </is>
       </c>
       <c r="N3" s="2" t="inlineStr">
@@ -706,18 +706,18 @@
       </c>
       <c r="J4" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K4" s="2" t="n">
         <v>1</v>
       </c>
       <c r="L4" s="2" t="n">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; TRD_003; MOFCOM_001; CASE_001; WB_001</t>
+          <t>MOFCOM_003; TRD_001; CASE_001; MOFCOM_001; TRD_003</t>
         </is>
       </c>
       <c r="N4" s="2" t="inlineStr">
@@ -774,18 +774,18 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>Operational Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K5" s="2" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="L5" s="2" t="n">
         <v>1</v>
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; TRD_003; CASE_007; WB_001; CASE_001</t>
+          <t>TRD_001; MOFCOM_004; MOFCOM_003; TRD_003; MOFCOM_006</t>
         </is>
       </c>
       <c r="N5" s="2" t="inlineStr">
@@ -842,7 +842,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K6" s="2" t="n">
@@ -853,7 +853,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; TRD_003; MOFCOM_001; CASE_001; WB_001</t>
+          <t>MOFCOM_003; TRD_001; MOFCOM_005; CASE_001; TRD_003</t>
         </is>
       </c>
       <c r="N6" s="2" t="inlineStr">
@@ -910,18 +910,18 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K7" s="2" t="n">
-        <v>1</v>
+        <v>0.667</v>
       </c>
       <c r="L7" s="2" t="n">
         <v>0.667</v>
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; MOFCOM_001; CASE_001; CASE_004; TRD_003</t>
+          <t>TRD_001; MOFCOM_003; CASE_004; MOFCOM_004; CASE_001</t>
         </is>
       </c>
       <c r="N7" s="2" t="inlineStr">
@@ -978,18 +978,18 @@
       </c>
       <c r="J8" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K8" s="2" t="n">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="L8" s="2" t="n">
         <v>0.667</v>
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; WB_001; MOFCOM_001; CASE_001; CASE_008</t>
+          <t>MOFCOM_003; TRD_001; WB_001; CASE_001; CASE_008</t>
         </is>
       </c>
       <c r="N8" s="2" t="inlineStr">
@@ -1046,18 +1046,18 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K9" s="2" t="n">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="L9" s="2" t="n">
         <v>0.667</v>
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>TRD_001; WB_001; CASE_001; MOFCOM_001; CASE_008</t>
+          <t>MOFCOM_003; TRD_001; WB_001; CASE_001; CASE_008</t>
         </is>
       </c>
       <c r="N9" s="2" t="inlineStr">
@@ -1125,7 +1125,7 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>SNE_001; CASE_010; CASE_001; CASE_008; WH_002</t>
+          <t>SNE_001; CASE_010; CASE_008; CASE_001; CASE_002</t>
         </is>
       </c>
       <c r="N10" s="2" t="inlineStr">
@@ -1193,7 +1193,7 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>SNE_001; CASE_010; CASE_001; CASE_008; TSLA_001</t>
+          <t>SNE_001; CASE_010; CASE_008; CASE_001; CASE_002</t>
         </is>
       </c>
       <c r="N11" s="2" t="inlineStr">
@@ -1261,7 +1261,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>SNE_001; CASE_010; CASE_008; CASE_001; EU_003</t>
+          <t>SNE_001; CASE_010; EU_003; CASE_008; CASE_001</t>
         </is>
       </c>
       <c r="N12" s="2" t="inlineStr">
@@ -1318,18 +1318,18 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K13" s="2" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="L13" s="2" t="n">
         <v>0.5</v>
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>CASE_010; CASE_003; TRD_001; WH_002; CASE_007</t>
+          <t>CASE_010; CASE_003; MOFCOM_004; CASE_007; TRD_001</t>
         </is>
       </c>
       <c r="N13" s="2" t="inlineStr">
@@ -1397,7 +1397,7 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>CASE_010; CASE_008; CASE_001; CASE_003; SNE_001</t>
+          <t>CASE_010; CASE_008; CASE_001; TSLA_001; SNE_001</t>
         </is>
       </c>
       <c r="N14" s="2" t="inlineStr">
@@ -1454,7 +1454,7 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K15" s="2" t="n">
@@ -1465,7 +1465,7 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; DHS_001; CASE_008; EU_003; SNE_001</t>
+          <t>DHS_001; CASE_001; MOFCOM_005; EU_003; CASE_008</t>
         </is>
       </c>
       <c r="N15" s="2" t="inlineStr">
@@ -1533,7 +1533,7 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>DHS_001; CASE_001; CASE_008; EU_003; CNGOV_001</t>
+          <t>DHS_001; CASE_001; MOFCOM_005; EU_003; CASE_008</t>
         </is>
       </c>
       <c r="N16" s="2" t="inlineStr">
@@ -1590,18 +1590,18 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K17" s="2" t="n">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="L17" s="2" t="n">
         <v>0.667</v>
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; DHS_001; EU_003; SNE_001; CASE_010</t>
+          <t>CASE_001; DHS_001; MOFCOM_004; MOFCOM_005; EU_003</t>
         </is>
       </c>
       <c r="N17" s="2" t="inlineStr">
@@ -1658,18 +1658,18 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Market Access Risk; Operational Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
+          <t>Market Access Risk; Operational Risk; Political Risk; Regulatory Risk; Supply Chain Risk; Trade Risk</t>
         </is>
       </c>
       <c r="K18" s="2" t="n">
-        <v>0.667</v>
+        <v>1</v>
       </c>
       <c r="L18" s="2" t="n">
         <v>0.333</v>
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>CASE_001; DHS_001; CASE_008; EU_003; SNE_001</t>
+          <t>DHS_001; CASE_001; MOFCOM_005; EU_003; CASE_008</t>
         </is>
       </c>
       <c r="N18" s="2" t="inlineStr">
@@ -1752,7 +1752,7 @@
         </is>
       </c>
       <c r="B4" s="2" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
@@ -1767,7 +1767,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.799</v>
+        <v>0.887</v>
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
@@ -1782,7 +1782,7 @@
         </is>
       </c>
       <c r="B6" s="2" t="n">
-        <v>0.681</v>
+        <v>0.701</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>

</xml_diff>